<commit_message>
Populate candidate pilot notes
</commit_message>
<xml_diff>
--- a/docs/challenge_set/pilot_worksheets.xlsx
+++ b/docs/challenge_set/pilot_worksheets.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R73a70816d68d4da2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Authoring" sheetId="2" r:id="R66898784d4fb428d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annotation" sheetId="3" r:id="R5d9b97651bec4b30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="4" r:id="R8a0476e162ac47fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" r:id="R5232b82c9c3c44ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R88e3b481414c49f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Authoring" sheetId="2" r:id="Rc9ccbbe0a4254137"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annotation" sheetId="3" r:id="Raa5c8d0c76164e3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="4" r:id="R62c6dd7c77c94d75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" r:id="R0aafa4963778400f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -84,7 +84,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -114,6 +114,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE8F5E9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF173A5A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBFE3F1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -183,7 +198,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="74">
+  <x:cellXfs count="82">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -332,6 +347,26 @@
     <x:xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -343,7 +378,7 @@
         <x:color rgb="FF1B5E20"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5E9"/>
         </x:patternFill>
       </x:fill>
@@ -353,7 +388,7 @@
         <x:color rgb="FF8B1E1E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -674,7 +709,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B3" s="29" t="str">
-        <x:v>Candidate pilot; excluded from reported results</x:v>
+        <x:v>Candidate pilot; 20 delegated synthetic notes accepted for publication; human annotation pending; excluded from reported results</x:v>
       </x:c>
       <x:c r="C3" s="27"/>
       <x:c r="D3" s="28" t="str">
@@ -682,7 +717,7 @@
       </x:c>
       <x:c r="E3" s="71" t="n">
         <x:f>COUNTIF('Authoring'!$E$2:$E$21,"&lt;&gt;")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F3" s="27"/>
       <x:c r="G3" s="27"/>
@@ -701,7 +736,7 @@
       </x:c>
       <x:c r="E4" s="72" t="n">
         <x:f>COUNTIF('Authoring'!$Q$2:$Q$21,"ready")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F4" s="27"/>
       <x:c r="G4" s="27"/>
@@ -720,7 +755,7 @@
       </x:c>
       <x:c r="E5" s="72" t="n">
         <x:f>COUNTIF('Authoring'!$K$2:$K$21,"yes")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F5" s="27"/>
       <x:c r="G5" s="27"/>
@@ -731,7 +766,7 @@
         <x:v>Passes</x:v>
       </x:c>
       <x:c r="B6" s="31" t="str">
-        <x:v>Two self-annotation passes, 7–14 days apart</x:v>
+        <x:v>Human annotation pass 1 and repeat pass remain pending</x:v>
       </x:c>
       <x:c r="C6" s="27"/>
       <x:c r="D6" s="32" t="str">
@@ -739,7 +774,7 @@
       </x:c>
       <x:c r="E6" s="73" t="n">
         <x:f>COUNTIF('Authoring'!$J$2:$J$21,"yes")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F6" s="27"/>
       <x:c r="G6" s="27"/>
@@ -750,7 +785,7 @@
         <x:v>Independent annotation</x:v>
       </x:c>
       <x:c r="B7" s="31" t="str">
-        <x:v>Not yet available; E1 remains incomplete</x:v>
+        <x:v>Not available; E1 remains incomplete</x:v>
       </x:c>
       <x:c r="C7" s="27"/>
       <x:c r="D7" s="27"/>
@@ -814,7 +849,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B12" s="36" t="str">
-        <x:v>Write or approve one original note in every Authoring row. Do not copy private, company, customer, school, or restricted text.</x:v>
+        <x:v>Twenty original synthetic notes are accepted for candidate-pilot publication under Ayo Adetayo's explicit protocol-level delegation; no direct note-level review was performed.</x:v>
       </x:c>
       <x:c r="C12" s="36"/>
       <x:c r="D12" s="36"/>
@@ -828,7 +863,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="38" t="str">
-        <x:v>Complete the rights, privacy, and predicate-family columns until Ready reads ready.</x:v>
+        <x:v>Rights, privacy, lineage, and predicate-family fields are complete; every Ready cell should read ready.</x:v>
       </x:c>
       <x:c r="C13" s="38"/>
       <x:c r="D13" s="38"/>
@@ -842,7 +877,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B14" s="38" t="str">
-        <x:v>Use a separate copy of the Annotation sheet for pass 1. Store it away before the washout.</x:v>
+        <x:v>Leave Annotation blank until a human completes pass 1 without viewing model output.</x:v>
       </x:c>
       <x:c r="C14" s="38"/>
       <x:c r="D14" s="38"/>
@@ -856,7 +891,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B15" s="38" t="str">
-        <x:v>After 7–14 days, shuffle record order and use a clean copy for pass 2 without opening pass 1.</x:v>
+        <x:v>After 7–14 days, the same human annotator uses a shuffled clean copy for pass 2 without opening pass 1.</x:v>
       </x:c>
       <x:c r="C15" s="38"/>
       <x:c r="D15" s="38"/>
@@ -884,7 +919,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B17" s="40" t="str">
-        <x:v>Do not call this independent agreement, adjudication, gold data, or a frozen set.</x:v>
+        <x:v>Do not call this independent agreement, adjudication, gold data, a frozen set, or operational-domain evidence.</x:v>
       </x:c>
       <x:c r="C17" s="40"/>
       <x:c r="D17" s="40"/>
@@ -916,8 +951,8 @@
     <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="56" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
@@ -925,9 +960,9 @@
     <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="34" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="30" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="42" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -984,7 +1019,7 @@
         <x:v>ready</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="32" customHeight="1">
+    <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="52" t="str">
         <x:v>ops-pilot-001</x:v>
       </x:c>
@@ -997,36 +1032,48 @@
       <x:c r="D2" s="52" t="str">
         <x:v>customer_support</x:v>
       </x:c>
-      <x:c r="E2" s="53"/>
+      <x:c r="E2" s="53" t="str">
+        <x:v>The support agent emailed a reset link to the customer on Monday.</x:v>
+      </x:c>
       <x:c r="F2" s="54" t="str">
-        <x:v>verbal_predicate</x:v>
+        <x:v>verbal_predicate;temporal_circumstance</x:v>
       </x:c>
       <x:c r="G2" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H2" s="55"/>
+      <x:c r="H2" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I2" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J2" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K2" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L2" s="54" t="str">
         <x:v>ops-pilot-001</x:v>
       </x:c>
-      <x:c r="M2" s="54"/>
-      <x:c r="N2" s="54"/>
-      <x:c r="O2" s="54"/>
-      <x:c r="P2" s="54"/>
+      <x:c r="M2" s="54" t="str">
+        <x:v>email</x:v>
+      </x:c>
+      <x:c r="N2" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O2" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P2" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q2" s="52" t="str">
         <x:f>IF(AND(E2&lt;&gt;"",H2&lt;&gt;"",J2="yes",K2="yes",M2&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="52" t="str">
         <x:v>ops-pilot-002</x:v>
       </x:c>
@@ -1039,36 +1086,48 @@
       <x:c r="D3" s="52" t="str">
         <x:v>customer_support</x:v>
       </x:c>
-      <x:c r="E3" s="53"/>
+      <x:c r="E3" s="53" t="str">
+        <x:v>The supervisor's approval of the replacement on Tuesday.</x:v>
+      </x:c>
       <x:c r="F3" s="54" t="str">
-        <x:v>nominal_predicate</x:v>
+        <x:v>nominal_predicate;temporal_circumstance</x:v>
       </x:c>
       <x:c r="G3" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H3" s="55"/>
+      <x:c r="H3" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I3" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J3" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K3" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L3" s="54" t="str">
         <x:v>ops-pilot-002</x:v>
       </x:c>
-      <x:c r="M3" s="54"/>
-      <x:c r="N3" s="54"/>
-      <x:c r="O3" s="54"/>
-      <x:c r="P3" s="54"/>
+      <x:c r="M3" s="54" t="str">
+        <x:v>approve</x:v>
+      </x:c>
+      <x:c r="N3" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O3" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P3" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q3" s="52" t="str">
         <x:f>IF(AND(E3&lt;&gt;"",H3&lt;&gt;"",J3="yes",K3="yes",M3&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="52" t="str">
         <x:v>ops-pilot-003</x:v>
       </x:c>
@@ -1081,36 +1140,48 @@
       <x:c r="D4" s="52" t="str">
         <x:v>customer_support</x:v>
       </x:c>
-      <x:c r="E4" s="53"/>
+      <x:c r="E4" s="53" t="str">
+        <x:v>The agent did not refund the duplicate charge.</x:v>
+      </x:c>
       <x:c r="F4" s="54" t="str">
-        <x:v>negation</x:v>
+        <x:v>negated;verbal_predicate</x:v>
       </x:c>
       <x:c r="G4" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H4" s="55"/>
+      <x:c r="H4" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I4" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J4" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K4" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L4" s="54" t="str">
         <x:v>ops-pilot-003</x:v>
       </x:c>
-      <x:c r="M4" s="54"/>
-      <x:c r="N4" s="54"/>
-      <x:c r="O4" s="54"/>
-      <x:c r="P4" s="54"/>
+      <x:c r="M4" s="54" t="str">
+        <x:v>refund</x:v>
+      </x:c>
+      <x:c r="N4" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O4" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P4" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q4" s="52" t="str">
         <x:f>IF(AND(E4&lt;&gt;"",H4&lt;&gt;"",J4="yes",K4="yes",M4&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
       <x:c r="A5" s="52" t="str">
         <x:v>ops-pilot-004</x:v>
       </x:c>
@@ -1123,36 +1194,48 @@
       <x:c r="D5" s="52" t="str">
         <x:v>customer_support</x:v>
       </x:c>
-      <x:c r="E5" s="53"/>
+      <x:c r="E5" s="53" t="str">
+        <x:v>Support may reopen the case.</x:v>
+      </x:c>
       <x:c r="F5" s="54" t="str">
-        <x:v>possibility</x:v>
+        <x:v>possible;verbal_predicate</x:v>
       </x:c>
       <x:c r="G5" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H5" s="55"/>
+      <x:c r="H5" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I5" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J5" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K5" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L5" s="54" t="str">
         <x:v>ops-pilot-004</x:v>
       </x:c>
-      <x:c r="M5" s="54"/>
-      <x:c r="N5" s="54"/>
-      <x:c r="O5" s="54"/>
-      <x:c r="P5" s="54"/>
+      <x:c r="M5" s="54" t="str">
+        <x:v>reopen</x:v>
+      </x:c>
+      <x:c r="N5" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O5" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P5" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q5" s="52" t="str">
         <x:f>IF(AND(E5&lt;&gt;"",H5&lt;&gt;"",J5="yes",K5="yes",M5&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="36" customHeight="1">
       <x:c r="A6" s="52" t="str">
         <x:v>ops-pilot-005</x:v>
       </x:c>
@@ -1165,36 +1248,48 @@
       <x:c r="D6" s="52" t="str">
         <x:v>it_incident_change</x:v>
       </x:c>
-      <x:c r="E6" s="53"/>
+      <x:c r="E6" s="53" t="str">
+        <x:v>The database was restarted by the on-call engineer at 02:15 UTC.</x:v>
+      </x:c>
       <x:c r="F6" s="54" t="str">
-        <x:v>passive_voice</x:v>
+        <x:v>passive_voice;temporal_circumstance</x:v>
       </x:c>
       <x:c r="G6" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H6" s="55"/>
+      <x:c r="H6" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I6" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J6" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K6" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L6" s="54" t="str">
         <x:v>ops-pilot-005</x:v>
       </x:c>
-      <x:c r="M6" s="54"/>
-      <x:c r="N6" s="54"/>
-      <x:c r="O6" s="54"/>
-      <x:c r="P6" s="54"/>
+      <x:c r="M6" s="54" t="str">
+        <x:v>restart</x:v>
+      </x:c>
+      <x:c r="N6" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O6" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P6" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q6" s="52" t="str">
         <x:f>IF(AND(E6&lt;&gt;"",H6&lt;&gt;"",J6="yes",K6="yes",M6&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="36" customHeight="1">
       <x:c r="A7" s="52" t="str">
         <x:v>ops-pilot-006</x:v>
       </x:c>
@@ -1207,36 +1302,48 @@
       <x:c r="D7" s="52" t="str">
         <x:v>it_incident_change</x:v>
       </x:c>
-      <x:c r="E7" s="53"/>
+      <x:c r="E7" s="53" t="str">
+        <x:v>The monitor detected latency and opened a ticket.</x:v>
+      </x:c>
       <x:c r="F7" s="54" t="str">
-        <x:v>coordination</x:v>
+        <x:v>coordination;multiple_predicates</x:v>
       </x:c>
       <x:c r="G7" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H7" s="55"/>
+      <x:c r="H7" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I7" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J7" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K7" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L7" s="54" t="str">
         <x:v>ops-pilot-006</x:v>
       </x:c>
-      <x:c r="M7" s="54"/>
-      <x:c r="N7" s="54"/>
-      <x:c r="O7" s="54"/>
-      <x:c r="P7" s="54"/>
+      <x:c r="M7" s="54" t="str">
+        <x:v>detect;open</x:v>
+      </x:c>
+      <x:c r="N7" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O7" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P7" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q7" s="52" t="str">
         <x:f>IF(AND(E7&lt;&gt;"",H7&lt;&gt;"",J7="yes",K7="yes",M7&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="36" customHeight="1">
       <x:c r="A8" s="52" t="str">
         <x:v>ops-pilot-007</x:v>
       </x:c>
@@ -1249,36 +1356,48 @@
       <x:c r="D8" s="52" t="str">
         <x:v>it_incident_change</x:v>
       </x:c>
-      <x:c r="E8" s="53"/>
+      <x:c r="E8" s="53" t="str">
+        <x:v>If the patch fails, the engineer will restore the prior version.</x:v>
+      </x:c>
       <x:c r="F8" s="54" t="str">
-        <x:v>multiple_predicates</x:v>
+        <x:v>conditional;future;multiple_predicates</x:v>
       </x:c>
       <x:c r="G8" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H8" s="55"/>
+      <x:c r="H8" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I8" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J8" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K8" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L8" s="54" t="str">
         <x:v>ops-pilot-007</x:v>
       </x:c>
-      <x:c r="M8" s="54"/>
-      <x:c r="N8" s="54"/>
-      <x:c r="O8" s="54"/>
-      <x:c r="P8" s="54"/>
+      <x:c r="M8" s="54" t="str">
+        <x:v>fail;restore</x:v>
+      </x:c>
+      <x:c r="N8" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O8" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P8" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q8" s="52" t="str">
         <x:f>IF(AND(E8&lt;&gt;"",H8&lt;&gt;"",J8="yes",K8="yes",M8&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="36" customHeight="1">
       <x:c r="A9" s="52" t="str">
         <x:v>ops-pilot-008</x:v>
       </x:c>
@@ -1291,36 +1410,48 @@
       <x:c r="D9" s="52" t="str">
         <x:v>it_incident_change</x:v>
       </x:c>
-      <x:c r="E9" s="53"/>
+      <x:c r="E9" s="53" t="str">
+        <x:v>The team lead reported that the service might degrade overnight.</x:v>
+      </x:c>
       <x:c r="F9" s="54" t="str">
-        <x:v>reported_event</x:v>
+        <x:v>reported;possible;multiple_predicates</x:v>
       </x:c>
       <x:c r="G9" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H9" s="55"/>
+      <x:c r="H9" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I9" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J9" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K9" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L9" s="54" t="str">
         <x:v>ops-pilot-008</x:v>
       </x:c>
-      <x:c r="M9" s="54"/>
-      <x:c r="N9" s="54"/>
-      <x:c r="O9" s="54"/>
-      <x:c r="P9" s="54"/>
+      <x:c r="M9" s="54" t="str">
+        <x:v>report;degrade</x:v>
+      </x:c>
+      <x:c r="N9" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O9" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P9" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q9" s="52" t="str">
         <x:f>IF(AND(E9&lt;&gt;"",H9&lt;&gt;"",J9="yes",K9="yes",M9&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="36" customHeight="1">
       <x:c r="A10" s="52" t="str">
         <x:v>ops-pilot-009</x:v>
       </x:c>
@@ -1333,36 +1464,48 @@
       <x:c r="D10" s="52" t="str">
         <x:v>billing_approvals</x:v>
       </x:c>
-      <x:c r="E10" s="53"/>
+      <x:c r="E10" s="53" t="str">
+        <x:v>The billing team's approval of the credit for the disputed fee.</x:v>
+      </x:c>
       <x:c r="F10" s="54" t="str">
-        <x:v>nominal_predicate;light_verb_ambiguity</x:v>
+        <x:v>nominal_predicate</x:v>
       </x:c>
       <x:c r="G10" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H10" s="55"/>
+      <x:c r="H10" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I10" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J10" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K10" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L10" s="54" t="str">
         <x:v>ops-pilot-009</x:v>
       </x:c>
-      <x:c r="M10" s="54"/>
-      <x:c r="N10" s="54"/>
-      <x:c r="O10" s="54"/>
-      <x:c r="P10" s="54"/>
+      <x:c r="M10" s="54" t="str">
+        <x:v>approve</x:v>
+      </x:c>
+      <x:c r="N10" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O10" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P10" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q10" s="52" t="str">
         <x:f>IF(AND(E10&lt;&gt;"",H10&lt;&gt;"",J10="yes",K10="yes",M10&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="36" customHeight="1">
       <x:c r="A11" s="52" t="str">
         <x:v>ops-pilot-010</x:v>
       </x:c>
@@ -1375,36 +1518,48 @@
       <x:c r="D11" s="52" t="str">
         <x:v>billing_approvals</x:v>
       </x:c>
-      <x:c r="E11" s="53"/>
+      <x:c r="E11" s="53" t="str">
+        <x:v>The invoice was not authorized by the reviewer.</x:v>
+      </x:c>
       <x:c r="F11" s="54" t="str">
-        <x:v>negation</x:v>
+        <x:v>negated;passive_voice</x:v>
       </x:c>
       <x:c r="G11" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H11" s="55"/>
+      <x:c r="H11" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I11" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J11" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K11" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L11" s="54" t="str">
         <x:v>ops-pilot-010</x:v>
       </x:c>
-      <x:c r="M11" s="54"/>
-      <x:c r="N11" s="54"/>
-      <x:c r="O11" s="54"/>
-      <x:c r="P11" s="54"/>
+      <x:c r="M11" s="54" t="str">
+        <x:v>authorize</x:v>
+      </x:c>
+      <x:c r="N11" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O11" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P11" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q11" s="52" t="str">
         <x:f>IF(AND(E11&lt;&gt;"",H11&lt;&gt;"",J11="yes",K11="yes",M11&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="36" customHeight="1">
       <x:c r="A12" s="52" t="str">
         <x:v>ops-pilot-011</x:v>
       </x:c>
@@ -1417,36 +1572,48 @@
       <x:c r="D12" s="52" t="str">
         <x:v>billing_approvals</x:v>
       </x:c>
-      <x:c r="E12" s="53"/>
+      <x:c r="E12" s="53" t="str">
+        <x:v>Procurement plans to renew the contract in June.</x:v>
+      </x:c>
       <x:c r="F12" s="54" t="str">
-        <x:v>planned_event</x:v>
+        <x:v>planned;multiple_predicates;temporal_circumstance</x:v>
       </x:c>
       <x:c r="G12" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H12" s="55"/>
+      <x:c r="H12" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I12" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J12" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K12" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L12" s="54" t="str">
         <x:v>ops-pilot-011</x:v>
       </x:c>
-      <x:c r="M12" s="54"/>
-      <x:c r="N12" s="54"/>
-      <x:c r="O12" s="54"/>
-      <x:c r="P12" s="54"/>
+      <x:c r="M12" s="54" t="str">
+        <x:v>plan;renew</x:v>
+      </x:c>
+      <x:c r="N12" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O12" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P12" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q12" s="52" t="str">
         <x:f>IF(AND(E12&lt;&gt;"",H12&lt;&gt;"",J12="yes",K12="yes",M12&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="36" customHeight="1">
       <x:c r="A13" s="52" t="str">
         <x:v>ops-pilot-012</x:v>
       </x:c>
@@ -1459,36 +1626,48 @@
       <x:c r="D13" s="52" t="str">
         <x:v>billing_approvals</x:v>
       </x:c>
-      <x:c r="E13" s="53"/>
+      <x:c r="E13" s="53" t="str">
+        <x:v>The reviewer, after the second audit, approved the revised amount.</x:v>
+      </x:c>
       <x:c r="F13" s="54" t="str">
-        <x:v>long_distance_argument</x:v>
+        <x:v>long_distance_argument;nominal_predicate;temporal_circumstance</x:v>
       </x:c>
       <x:c r="G13" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H13" s="55"/>
+      <x:c r="H13" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I13" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J13" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K13" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L13" s="54" t="str">
         <x:v>ops-pilot-012</x:v>
       </x:c>
-      <x:c r="M13" s="54"/>
-      <x:c r="N13" s="54"/>
-      <x:c r="O13" s="54"/>
-      <x:c r="P13" s="54"/>
+      <x:c r="M13" s="54" t="str">
+        <x:v>audit;approve</x:v>
+      </x:c>
+      <x:c r="N13" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O13" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P13" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q13" s="52" t="str">
         <x:f>IF(AND(E13&lt;&gt;"",H13&lt;&gt;"",J13="yes",K13="yes",M13&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="36" customHeight="1">
       <x:c r="A14" s="52" t="str">
         <x:v>ops-pilot-013</x:v>
       </x:c>
@@ -1501,36 +1680,48 @@
       <x:c r="D14" s="52" t="str">
         <x:v>logistics_fulfillment</x:v>
       </x:c>
-      <x:c r="E14" s="53"/>
+      <x:c r="E14" s="53" t="str">
+        <x:v>The parcel was packed by warehouse staff before noon.</x:v>
+      </x:c>
       <x:c r="F14" s="54" t="str">
-        <x:v>passive_voice</x:v>
+        <x:v>passive_voice;temporal_circumstance</x:v>
       </x:c>
       <x:c r="G14" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H14" s="55"/>
+      <x:c r="H14" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I14" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J14" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K14" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L14" s="54" t="str">
         <x:v>ops-pilot-013</x:v>
       </x:c>
-      <x:c r="M14" s="54"/>
-      <x:c r="N14" s="54"/>
-      <x:c r="O14" s="54"/>
-      <x:c r="P14" s="54"/>
+      <x:c r="M14" s="54" t="str">
+        <x:v>pack</x:v>
+      </x:c>
+      <x:c r="N14" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O14" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P14" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q14" s="52" t="str">
         <x:f>IF(AND(E14&lt;&gt;"",H14&lt;&gt;"",J14="yes",K14="yes",M14&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="36" customHeight="1">
       <x:c r="A15" s="52" t="str">
         <x:v>ops-pilot-014</x:v>
       </x:c>
@@ -1543,36 +1734,48 @@
       <x:c r="D15" s="52" t="str">
         <x:v>logistics_fulfillment</x:v>
       </x:c>
-      <x:c r="E15" s="53"/>
+      <x:c r="E15" s="53" t="str">
+        <x:v>The dispatcher assigned the route and notified the courier.</x:v>
+      </x:c>
       <x:c r="F15" s="54" t="str">
-        <x:v>coordination</x:v>
+        <x:v>coordination;multiple_predicates</x:v>
       </x:c>
       <x:c r="G15" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H15" s="55"/>
+      <x:c r="H15" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I15" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J15" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K15" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L15" s="54" t="str">
         <x:v>ops-pilot-014</x:v>
       </x:c>
-      <x:c r="M15" s="54"/>
-      <x:c r="N15" s="54"/>
-      <x:c r="O15" s="54"/>
-      <x:c r="P15" s="54"/>
+      <x:c r="M15" s="54" t="str">
+        <x:v>assign;notify</x:v>
+      </x:c>
+      <x:c r="N15" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O15" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P15" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q15" s="52" t="str">
         <x:f>IF(AND(E15&lt;&gt;"",H15&lt;&gt;"",J15="yes",K15="yes",M15&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="36" customHeight="1">
       <x:c r="A16" s="52" t="str">
         <x:v>ops-pilot-015</x:v>
       </x:c>
@@ -1585,36 +1788,48 @@
       <x:c r="D16" s="52" t="str">
         <x:v>logistics_fulfillment</x:v>
       </x:c>
-      <x:c r="E16" s="53"/>
+      <x:c r="E16" s="53" t="str">
+        <x:v>The carrier will deliver the shipment after sunrise.</x:v>
+      </x:c>
       <x:c r="F16" s="54" t="str">
-        <x:v>temporal_circumstance</x:v>
+        <x:v>future;temporal_circumstance</x:v>
       </x:c>
       <x:c r="G16" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H16" s="55"/>
+      <x:c r="H16" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I16" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J16" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K16" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L16" s="54" t="str">
         <x:v>ops-pilot-015</x:v>
       </x:c>
-      <x:c r="M16" s="54"/>
-      <x:c r="N16" s="54"/>
-      <x:c r="O16" s="54"/>
-      <x:c r="P16" s="54"/>
+      <x:c r="M16" s="54" t="str">
+        <x:v>deliver</x:v>
+      </x:c>
+      <x:c r="N16" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O16" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P16" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q16" s="52" t="str">
         <x:f>IF(AND(E16&lt;&gt;"",H16&lt;&gt;"",J16="yes",K16="yes",M16&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="36" customHeight="1">
       <x:c r="A17" s="52" t="str">
         <x:v>ops-pilot-016</x:v>
       </x:c>
@@ -1627,36 +1842,48 @@
       <x:c r="D17" s="52" t="str">
         <x:v>logistics_fulfillment</x:v>
       </x:c>
-      <x:c r="E17" s="53"/>
+      <x:c r="E17" s="53" t="str">
+        <x:v>The delivery address remains on the label.</x:v>
+      </x:c>
       <x:c r="F17" s="54" t="str">
         <x:v>non_eventive_nominal</x:v>
       </x:c>
       <x:c r="G17" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H17" s="55"/>
+      <x:c r="H17" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I17" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J17" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K17" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L17" s="54" t="str">
         <x:v>ops-pilot-016</x:v>
       </x:c>
-      <x:c r="M17" s="54"/>
-      <x:c r="N17" s="54"/>
-      <x:c r="O17" s="54"/>
-      <x:c r="P17" s="54"/>
+      <x:c r="M17" s="54" t="str">
+        <x:v>delivery_non_eventive</x:v>
+      </x:c>
+      <x:c r="N17" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O17" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P17" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q17" s="52" t="str">
         <x:f>IF(AND(E17&lt;&gt;"",H17&lt;&gt;"",J17="yes",K17="yes",M17&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="36" customHeight="1">
       <x:c r="A18" s="52" t="str">
         <x:v>ops-pilot-017</x:v>
       </x:c>
@@ -1669,36 +1896,48 @@
       <x:c r="D18" s="52" t="str">
         <x:v>project_administration</x:v>
       </x:c>
-      <x:c r="E18" s="53"/>
+      <x:c r="E18" s="53" t="str">
+        <x:v>Following the committee's approval of the agenda, the coordinator scheduled the planned review.</x:v>
+      </x:c>
       <x:c r="F18" s="54" t="str">
-        <x:v>nominal_predicate</x:v>
+        <x:v>nominal_predicate;planned;multiple_predicates;temporal_circumstance</x:v>
       </x:c>
       <x:c r="G18" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H18" s="55"/>
+      <x:c r="H18" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I18" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J18" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K18" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L18" s="54" t="str">
         <x:v>ops-pilot-017</x:v>
       </x:c>
-      <x:c r="M18" s="54"/>
-      <x:c r="N18" s="54"/>
-      <x:c r="O18" s="54"/>
-      <x:c r="P18" s="54"/>
+      <x:c r="M18" s="54" t="str">
+        <x:v>approve;schedule;review</x:v>
+      </x:c>
+      <x:c r="N18" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O18" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P18" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q18" s="52" t="str">
         <x:f>IF(AND(E18&lt;&gt;"",H18&lt;&gt;"",J18="yes",K18="yes",M18&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="36" customHeight="1">
       <x:c r="A19" s="52" t="str">
         <x:v>ops-pilot-018</x:v>
       </x:c>
@@ -1711,36 +1950,48 @@
       <x:c r="D19" s="52" t="str">
         <x:v>project_administration</x:v>
       </x:c>
-      <x:c r="E19" s="53"/>
+      <x:c r="E19" s="53" t="str">
+        <x:v>The project lead said that the team must revise the schedule.</x:v>
+      </x:c>
       <x:c r="F19" s="54" t="str">
-        <x:v>reported_event</x:v>
+        <x:v>reported;necessary;multiple_predicates;non_eventive_nominal</x:v>
       </x:c>
       <x:c r="G19" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H19" s="55"/>
+      <x:c r="H19" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I19" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J19" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K19" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L19" s="54" t="str">
         <x:v>ops-pilot-018</x:v>
       </x:c>
-      <x:c r="M19" s="54"/>
-      <x:c r="N19" s="54"/>
-      <x:c r="O19" s="54"/>
-      <x:c r="P19" s="54"/>
+      <x:c r="M19" s="54" t="str">
+        <x:v>say;revise;schedule_non_eventive</x:v>
+      </x:c>
+      <x:c r="N19" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O19" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P19" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q19" s="52" t="str">
         <x:f>IF(AND(E19&lt;&gt;"",H19&lt;&gt;"",J19="yes",K19="yes",M19&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="36" customHeight="1">
       <x:c r="A20" s="52" t="str">
         <x:v>ops-pilot-019</x:v>
       </x:c>
@@ -1753,36 +2004,48 @@
       <x:c r="D20" s="52" t="str">
         <x:v>project_administration</x:v>
       </x:c>
-      <x:c r="E20" s="53"/>
+      <x:c r="E20" s="53" t="str">
+        <x:v>Would the committee postpone the review if the chair were unavailable?</x:v>
+      </x:c>
       <x:c r="F20" s="54" t="str">
-        <x:v>hypothetical_or_questioned</x:v>
+        <x:v>hypothetical;conditional;questioned;nominal_predicate</x:v>
       </x:c>
       <x:c r="G20" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H20" s="55"/>
+      <x:c r="H20" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I20" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J20" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K20" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L20" s="54" t="str">
         <x:v>ops-pilot-019</x:v>
       </x:c>
-      <x:c r="M20" s="54"/>
-      <x:c r="N20" s="54"/>
-      <x:c r="O20" s="54"/>
-      <x:c r="P20" s="54"/>
+      <x:c r="M20" s="54" t="str">
+        <x:v>postpone;review</x:v>
+      </x:c>
+      <x:c r="N20" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O20" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P20" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q20" s="52" t="str">
         <x:f>IF(AND(E20&lt;&gt;"",H20&lt;&gt;"",J20="yes",K20="yes",M20&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="32" customHeight="1">
+        <x:v>ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="36" customHeight="1">
       <x:c r="A21" s="52" t="str">
         <x:v>ops-pilot-020</x:v>
       </x:c>
@@ -1795,33 +2058,45 @@
       <x:c r="D21" s="52" t="str">
         <x:v>project_administration</x:v>
       </x:c>
-      <x:c r="E21" s="53"/>
+      <x:c r="E21" s="53" t="str">
+        <x:v>The administrator did not schedule the review that the committee requested for next week.</x:v>
+      </x:c>
       <x:c r="F21" s="54" t="str">
-        <x:v>embedded_argument</x:v>
+        <x:v>negated;embedded_argument;long_distance_argument;multiple_predicates;nominal_predicate</x:v>
       </x:c>
       <x:c r="G21" s="54" t="str">
         <x:v>Ayo Adetayo</x:v>
       </x:c>
-      <x:c r="H21" s="55"/>
+      <x:c r="H21" s="55" t="n">
+        <x:v>46243</x:v>
+      </x:c>
       <x:c r="I21" s="54" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
       <x:c r="J21" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="K21" s="54" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L21" s="54" t="str">
         <x:v>ops-pilot-020</x:v>
       </x:c>
-      <x:c r="M21" s="54"/>
-      <x:c r="N21" s="54"/>
-      <x:c r="O21" s="54"/>
-      <x:c r="P21" s="54"/>
+      <x:c r="M21" s="54" t="str">
+        <x:v>schedule;review;request</x:v>
+      </x:c>
+      <x:c r="N21" s="54" t="str">
+        <x:v>Original synthetic note; no external source.</x:v>
+      </x:c>
+      <x:c r="O21" s="54" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="P21" s="54" t="str">
+        <x:v>Accepted under explicit protocol-level delegation; no direct note-level review.</x:v>
+      </x:c>
       <x:c r="Q21" s="52" t="str">
         <x:f>IF(AND(E21&lt;&gt;"",H21&lt;&gt;"",J21="yes",K21="yes",M21&lt;&gt;""),"ready","incomplete")</x:f>
-        <x:v>incomplete</x:v>
+        <x:v>ready</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1845,7 +2120,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8df0b9f7a1e47ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31d1ba07c17a4714"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1883,6 +2158,7 @@
     <x:col min="27" max="27" width="18" hidden="0" customWidth="1"/>
     <x:col min="28" max="28" width="24" hidden="0" customWidth="1"/>
     <x:col min="29" max="29" width="36" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="44" customHeight="1">
@@ -1972,6 +2248,9 @@
       </x:c>
       <x:c r="AC1" s="51" t="str">
         <x:v>rationale</x:v>
+      </x:c>
+      <x:c r="AD1" s="78" t="str">
+        <x:v>qualifier_assessed</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
@@ -2004,6 +2283,7 @@
       <x:c r="AA2" s="54"/>
       <x:c r="AB2" s="54"/>
       <x:c r="AC2" s="54"/>
+      <x:c r="AD2" s="80"/>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="54"/>
@@ -2035,6 +2315,7 @@
       <x:c r="AA3" s="54"/>
       <x:c r="AB3" s="54"/>
       <x:c r="AC3" s="54"/>
+      <x:c r="AD3" s="81"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="54"/>
@@ -2066,6 +2347,7 @@
       <x:c r="AA4" s="54"/>
       <x:c r="AB4" s="54"/>
       <x:c r="AC4" s="54"/>
+      <x:c r="AD4" s="80"/>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="54"/>
@@ -2097,6 +2379,7 @@
       <x:c r="AA5" s="54"/>
       <x:c r="AB5" s="54"/>
       <x:c r="AC5" s="54"/>
+      <x:c r="AD5" s="81"/>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="54"/>
@@ -2128,6 +2411,7 @@
       <x:c r="AA6" s="54"/>
       <x:c r="AB6" s="54"/>
       <x:c r="AC6" s="54"/>
+      <x:c r="AD6" s="80"/>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="54"/>
@@ -2159,6 +2443,7 @@
       <x:c r="AA7" s="54"/>
       <x:c r="AB7" s="54"/>
       <x:c r="AC7" s="54"/>
+      <x:c r="AD7" s="81"/>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
       <x:c r="A8" s="54"/>
@@ -2190,6 +2475,7 @@
       <x:c r="AA8" s="54"/>
       <x:c r="AB8" s="54"/>
       <x:c r="AC8" s="54"/>
+      <x:c r="AD8" s="80"/>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" s="54"/>
@@ -2221,6 +2507,7 @@
       <x:c r="AA9" s="54"/>
       <x:c r="AB9" s="54"/>
       <x:c r="AC9" s="54"/>
+      <x:c r="AD9" s="81"/>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
       <x:c r="A10" s="54"/>
@@ -2252,6 +2539,7 @@
       <x:c r="AA10" s="54"/>
       <x:c r="AB10" s="54"/>
       <x:c r="AC10" s="54"/>
+      <x:c r="AD10" s="80"/>
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
       <x:c r="A11" s="54"/>
@@ -2283,6 +2571,7 @@
       <x:c r="AA11" s="54"/>
       <x:c r="AB11" s="54"/>
       <x:c r="AC11" s="54"/>
+      <x:c r="AD11" s="81"/>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
       <x:c r="A12" s="54"/>
@@ -2314,6 +2603,7 @@
       <x:c r="AA12" s="54"/>
       <x:c r="AB12" s="54"/>
       <x:c r="AC12" s="54"/>
+      <x:c r="AD12" s="80"/>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
       <x:c r="A13" s="54"/>
@@ -2345,6 +2635,7 @@
       <x:c r="AA13" s="54"/>
       <x:c r="AB13" s="54"/>
       <x:c r="AC13" s="54"/>
+      <x:c r="AD13" s="81"/>
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
       <x:c r="A14" s="54"/>
@@ -2376,6 +2667,7 @@
       <x:c r="AA14" s="54"/>
       <x:c r="AB14" s="54"/>
       <x:c r="AC14" s="54"/>
+      <x:c r="AD14" s="80"/>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
       <x:c r="A15" s="54"/>
@@ -2407,6 +2699,7 @@
       <x:c r="AA15" s="54"/>
       <x:c r="AB15" s="54"/>
       <x:c r="AC15" s="54"/>
+      <x:c r="AD15" s="81"/>
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
       <x:c r="A16" s="54"/>
@@ -2438,6 +2731,7 @@
       <x:c r="AA16" s="54"/>
       <x:c r="AB16" s="54"/>
       <x:c r="AC16" s="54"/>
+      <x:c r="AD16" s="80"/>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
       <x:c r="A17" s="54"/>
@@ -2469,6 +2763,7 @@
       <x:c r="AA17" s="54"/>
       <x:c r="AB17" s="54"/>
       <x:c r="AC17" s="54"/>
+      <x:c r="AD17" s="81"/>
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
       <x:c r="A18" s="54"/>
@@ -2500,6 +2795,7 @@
       <x:c r="AA18" s="54"/>
       <x:c r="AB18" s="54"/>
       <x:c r="AC18" s="54"/>
+      <x:c r="AD18" s="80"/>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
       <x:c r="A19" s="54"/>
@@ -2531,6 +2827,7 @@
       <x:c r="AA19" s="54"/>
       <x:c r="AB19" s="54"/>
       <x:c r="AC19" s="54"/>
+      <x:c r="AD19" s="81"/>
     </x:row>
     <x:row r="20" ht="28" customHeight="1">
       <x:c r="A20" s="54"/>
@@ -2562,6 +2859,7 @@
       <x:c r="AA20" s="54"/>
       <x:c r="AB20" s="54"/>
       <x:c r="AC20" s="54"/>
+      <x:c r="AD20" s="80"/>
     </x:row>
     <x:row r="21" ht="28" customHeight="1">
       <x:c r="A21" s="54"/>
@@ -2593,6 +2891,7 @@
       <x:c r="AA21" s="54"/>
       <x:c r="AB21" s="54"/>
       <x:c r="AC21" s="54"/>
+      <x:c r="AD21" s="81"/>
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
       <x:c r="A22" s="54"/>
@@ -2624,6 +2923,7 @@
       <x:c r="AA22" s="54"/>
       <x:c r="AB22" s="54"/>
       <x:c r="AC22" s="54"/>
+      <x:c r="AD22" s="80"/>
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
       <x:c r="A23" s="54"/>
@@ -2655,6 +2955,7 @@
       <x:c r="AA23" s="54"/>
       <x:c r="AB23" s="54"/>
       <x:c r="AC23" s="54"/>
+      <x:c r="AD23" s="81"/>
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
       <x:c r="A24" s="54"/>
@@ -2686,6 +2987,7 @@
       <x:c r="AA24" s="54"/>
       <x:c r="AB24" s="54"/>
       <x:c r="AC24" s="54"/>
+      <x:c r="AD24" s="80"/>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
       <x:c r="A25" s="54"/>
@@ -2717,6 +3019,7 @@
       <x:c r="AA25" s="54"/>
       <x:c r="AB25" s="54"/>
       <x:c r="AC25" s="54"/>
+      <x:c r="AD25" s="81"/>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="54"/>
@@ -2748,6 +3051,7 @@
       <x:c r="AA26" s="54"/>
       <x:c r="AB26" s="54"/>
       <x:c r="AC26" s="54"/>
+      <x:c r="AD26" s="80"/>
     </x:row>
     <x:row r="27" ht="28" customHeight="1">
       <x:c r="A27" s="54"/>
@@ -2779,6 +3083,7 @@
       <x:c r="AA27" s="54"/>
       <x:c r="AB27" s="54"/>
       <x:c r="AC27" s="54"/>
+      <x:c r="AD27" s="81"/>
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
       <x:c r="A28" s="54"/>
@@ -2810,6 +3115,7 @@
       <x:c r="AA28" s="54"/>
       <x:c r="AB28" s="54"/>
       <x:c r="AC28" s="54"/>
+      <x:c r="AD28" s="80"/>
     </x:row>
     <x:row r="29" ht="28" customHeight="1">
       <x:c r="A29" s="54"/>
@@ -2841,6 +3147,7 @@
       <x:c r="AA29" s="54"/>
       <x:c r="AB29" s="54"/>
       <x:c r="AC29" s="54"/>
+      <x:c r="AD29" s="81"/>
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
       <x:c r="A30" s="54"/>
@@ -2872,6 +3179,7 @@
       <x:c r="AA30" s="54"/>
       <x:c r="AB30" s="54"/>
       <x:c r="AC30" s="54"/>
+      <x:c r="AD30" s="80"/>
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="54"/>
@@ -2903,6 +3211,7 @@
       <x:c r="AA31" s="54"/>
       <x:c r="AB31" s="54"/>
       <x:c r="AC31" s="54"/>
+      <x:c r="AD31" s="81"/>
     </x:row>
     <x:row r="32" ht="28" customHeight="1">
       <x:c r="A32" s="54"/>
@@ -2934,6 +3243,7 @@
       <x:c r="AA32" s="54"/>
       <x:c r="AB32" s="54"/>
       <x:c r="AC32" s="54"/>
+      <x:c r="AD32" s="80"/>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="54"/>
@@ -2965,6 +3275,7 @@
       <x:c r="AA33" s="54"/>
       <x:c r="AB33" s="54"/>
       <x:c r="AC33" s="54"/>
+      <x:c r="AD33" s="81"/>
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
       <x:c r="A34" s="54"/>
@@ -2996,6 +3307,7 @@
       <x:c r="AA34" s="54"/>
       <x:c r="AB34" s="54"/>
       <x:c r="AC34" s="54"/>
+      <x:c r="AD34" s="80"/>
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
       <x:c r="A35" s="54"/>
@@ -3027,6 +3339,7 @@
       <x:c r="AA35" s="54"/>
       <x:c r="AB35" s="54"/>
       <x:c r="AC35" s="54"/>
+      <x:c r="AD35" s="81"/>
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
       <x:c r="A36" s="54"/>
@@ -3058,6 +3371,7 @@
       <x:c r="AA36" s="54"/>
       <x:c r="AB36" s="54"/>
       <x:c r="AC36" s="54"/>
+      <x:c r="AD36" s="80"/>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
       <x:c r="A37" s="54"/>
@@ -3089,6 +3403,7 @@
       <x:c r="AA37" s="54"/>
       <x:c r="AB37" s="54"/>
       <x:c r="AC37" s="54"/>
+      <x:c r="AD37" s="81"/>
     </x:row>
     <x:row r="38" ht="28" customHeight="1">
       <x:c r="A38" s="54"/>
@@ -3120,6 +3435,7 @@
       <x:c r="AA38" s="54"/>
       <x:c r="AB38" s="54"/>
       <x:c r="AC38" s="54"/>
+      <x:c r="AD38" s="80"/>
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
       <x:c r="A39" s="54"/>
@@ -3151,6 +3467,7 @@
       <x:c r="AA39" s="54"/>
       <x:c r="AB39" s="54"/>
       <x:c r="AC39" s="54"/>
+      <x:c r="AD39" s="81"/>
     </x:row>
     <x:row r="40" ht="28" customHeight="1">
       <x:c r="A40" s="54"/>
@@ -3182,6 +3499,7 @@
       <x:c r="AA40" s="54"/>
       <x:c r="AB40" s="54"/>
       <x:c r="AC40" s="54"/>
+      <x:c r="AD40" s="80"/>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="54"/>
@@ -3213,6 +3531,7 @@
       <x:c r="AA41" s="54"/>
       <x:c r="AB41" s="54"/>
       <x:c r="AC41" s="54"/>
+      <x:c r="AD41" s="81"/>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
       <x:c r="A42" s="54"/>
@@ -3244,6 +3563,7 @@
       <x:c r="AA42" s="54"/>
       <x:c r="AB42" s="54"/>
       <x:c r="AC42" s="54"/>
+      <x:c r="AD42" s="80"/>
     </x:row>
     <x:row r="43" ht="28" customHeight="1">
       <x:c r="A43" s="54"/>
@@ -3275,6 +3595,7 @@
       <x:c r="AA43" s="54"/>
       <x:c r="AB43" s="54"/>
       <x:c r="AC43" s="54"/>
+      <x:c r="AD43" s="81"/>
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="54"/>
@@ -3306,6 +3627,7 @@
       <x:c r="AA44" s="54"/>
       <x:c r="AB44" s="54"/>
       <x:c r="AC44" s="54"/>
+      <x:c r="AD44" s="80"/>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
       <x:c r="A45" s="54"/>
@@ -3337,6 +3659,7 @@
       <x:c r="AA45" s="54"/>
       <x:c r="AB45" s="54"/>
       <x:c r="AC45" s="54"/>
+      <x:c r="AD45" s="81"/>
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
       <x:c r="A46" s="54"/>
@@ -3368,6 +3691,7 @@
       <x:c r="AA46" s="54"/>
       <x:c r="AB46" s="54"/>
       <x:c r="AC46" s="54"/>
+      <x:c r="AD46" s="80"/>
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
       <x:c r="A47" s="54"/>
@@ -3399,6 +3723,7 @@
       <x:c r="AA47" s="54"/>
       <x:c r="AB47" s="54"/>
       <x:c r="AC47" s="54"/>
+      <x:c r="AD47" s="81"/>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
       <x:c r="A48" s="54"/>
@@ -3430,6 +3755,7 @@
       <x:c r="AA48" s="54"/>
       <x:c r="AB48" s="54"/>
       <x:c r="AC48" s="54"/>
+      <x:c r="AD48" s="80"/>
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
       <x:c r="A49" s="54"/>
@@ -3461,6 +3787,7 @@
       <x:c r="AA49" s="54"/>
       <x:c r="AB49" s="54"/>
       <x:c r="AC49" s="54"/>
+      <x:c r="AD49" s="81"/>
     </x:row>
     <x:row r="50" ht="28" customHeight="1">
       <x:c r="A50" s="54"/>
@@ -3492,6 +3819,7 @@
       <x:c r="AA50" s="54"/>
       <x:c r="AB50" s="54"/>
       <x:c r="AC50" s="54"/>
+      <x:c r="AD50" s="80"/>
     </x:row>
     <x:row r="51" ht="28" customHeight="1">
       <x:c r="A51" s="54"/>
@@ -3523,6 +3851,7 @@
       <x:c r="AA51" s="54"/>
       <x:c r="AB51" s="54"/>
       <x:c r="AC51" s="54"/>
+      <x:c r="AD51" s="81"/>
     </x:row>
     <x:row r="52" ht="28" customHeight="1">
       <x:c r="A52" s="54"/>
@@ -3554,6 +3883,7 @@
       <x:c r="AA52" s="54"/>
       <x:c r="AB52" s="54"/>
       <x:c r="AC52" s="54"/>
+      <x:c r="AD52" s="80"/>
     </x:row>
     <x:row r="53" ht="28" customHeight="1">
       <x:c r="A53" s="54"/>
@@ -3585,6 +3915,7 @@
       <x:c r="AA53" s="54"/>
       <x:c r="AB53" s="54"/>
       <x:c r="AC53" s="54"/>
+      <x:c r="AD53" s="81"/>
     </x:row>
     <x:row r="54" ht="28" customHeight="1">
       <x:c r="A54" s="54"/>
@@ -3616,6 +3947,7 @@
       <x:c r="AA54" s="54"/>
       <x:c r="AB54" s="54"/>
       <x:c r="AC54" s="54"/>
+      <x:c r="AD54" s="80"/>
     </x:row>
     <x:row r="55" ht="28" customHeight="1">
       <x:c r="A55" s="54"/>
@@ -3647,6 +3979,7 @@
       <x:c r="AA55" s="54"/>
       <x:c r="AB55" s="54"/>
       <x:c r="AC55" s="54"/>
+      <x:c r="AD55" s="81"/>
     </x:row>
     <x:row r="56" ht="28" customHeight="1">
       <x:c r="A56" s="54"/>
@@ -3678,6 +4011,7 @@
       <x:c r="AA56" s="54"/>
       <x:c r="AB56" s="54"/>
       <x:c r="AC56" s="54"/>
+      <x:c r="AD56" s="80"/>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
       <x:c r="A57" s="54"/>
@@ -3709,6 +4043,7 @@
       <x:c r="AA57" s="54"/>
       <x:c r="AB57" s="54"/>
       <x:c r="AC57" s="54"/>
+      <x:c r="AD57" s="81"/>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
       <x:c r="A58" s="54"/>
@@ -3740,6 +4075,7 @@
       <x:c r="AA58" s="54"/>
       <x:c r="AB58" s="54"/>
       <x:c r="AC58" s="54"/>
+      <x:c r="AD58" s="80"/>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
       <x:c r="A59" s="54"/>
@@ -3771,6 +4107,7 @@
       <x:c r="AA59" s="54"/>
       <x:c r="AB59" s="54"/>
       <x:c r="AC59" s="54"/>
+      <x:c r="AD59" s="81"/>
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
       <x:c r="A60" s="54"/>
@@ -3802,6 +4139,7 @@
       <x:c r="AA60" s="54"/>
       <x:c r="AB60" s="54"/>
       <x:c r="AC60" s="54"/>
+      <x:c r="AD60" s="80"/>
     </x:row>
     <x:row r="61" ht="28" customHeight="1">
       <x:c r="A61" s="54"/>
@@ -3833,6 +4171,7 @@
       <x:c r="AA61" s="54"/>
       <x:c r="AB61" s="54"/>
       <x:c r="AC61" s="54"/>
+      <x:c r="AD61" s="81"/>
     </x:row>
     <x:row r="62" ht="28" customHeight="1">
       <x:c r="A62" s="54"/>
@@ -3864,6 +4203,7 @@
       <x:c r="AA62" s="54"/>
       <x:c r="AB62" s="54"/>
       <x:c r="AC62" s="54"/>
+      <x:c r="AD62" s="80"/>
     </x:row>
     <x:row r="63" ht="28" customHeight="1">
       <x:c r="A63" s="54"/>
@@ -3895,6 +4235,7 @@
       <x:c r="AA63" s="54"/>
       <x:c r="AB63" s="54"/>
       <x:c r="AC63" s="54"/>
+      <x:c r="AD63" s="81"/>
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
       <x:c r="A64" s="54"/>
@@ -3926,6 +4267,7 @@
       <x:c r="AA64" s="54"/>
       <x:c r="AB64" s="54"/>
       <x:c r="AC64" s="54"/>
+      <x:c r="AD64" s="80"/>
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
       <x:c r="A65" s="54"/>
@@ -3957,6 +4299,7 @@
       <x:c r="AA65" s="54"/>
       <x:c r="AB65" s="54"/>
       <x:c r="AC65" s="54"/>
+      <x:c r="AD65" s="81"/>
     </x:row>
     <x:row r="66" ht="28" customHeight="1">
       <x:c r="A66" s="54"/>
@@ -3988,6 +4331,7 @@
       <x:c r="AA66" s="54"/>
       <x:c r="AB66" s="54"/>
       <x:c r="AC66" s="54"/>
+      <x:c r="AD66" s="80"/>
     </x:row>
     <x:row r="67" ht="28" customHeight="1">
       <x:c r="A67" s="54"/>
@@ -4019,6 +4363,7 @@
       <x:c r="AA67" s="54"/>
       <x:c r="AB67" s="54"/>
       <x:c r="AC67" s="54"/>
+      <x:c r="AD67" s="81"/>
     </x:row>
     <x:row r="68" ht="28" customHeight="1">
       <x:c r="A68" s="54"/>
@@ -4050,6 +4395,7 @@
       <x:c r="AA68" s="54"/>
       <x:c r="AB68" s="54"/>
       <x:c r="AC68" s="54"/>
+      <x:c r="AD68" s="80"/>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
       <x:c r="A69" s="54"/>
@@ -4081,6 +4427,7 @@
       <x:c r="AA69" s="54"/>
       <x:c r="AB69" s="54"/>
       <x:c r="AC69" s="54"/>
+      <x:c r="AD69" s="81"/>
     </x:row>
     <x:row r="70" ht="28" customHeight="1">
       <x:c r="A70" s="54"/>
@@ -4112,6 +4459,7 @@
       <x:c r="AA70" s="54"/>
       <x:c r="AB70" s="54"/>
       <x:c r="AC70" s="54"/>
+      <x:c r="AD70" s="80"/>
     </x:row>
     <x:row r="71" ht="28" customHeight="1">
       <x:c r="A71" s="54"/>
@@ -4143,6 +4491,7 @@
       <x:c r="AA71" s="54"/>
       <x:c r="AB71" s="54"/>
       <x:c r="AC71" s="54"/>
+      <x:c r="AD71" s="81"/>
     </x:row>
     <x:row r="72" ht="28" customHeight="1">
       <x:c r="A72" s="54"/>
@@ -4174,6 +4523,7 @@
       <x:c r="AA72" s="54"/>
       <x:c r="AB72" s="54"/>
       <x:c r="AC72" s="54"/>
+      <x:c r="AD72" s="80"/>
     </x:row>
     <x:row r="73" ht="28" customHeight="1">
       <x:c r="A73" s="54"/>
@@ -4205,6 +4555,7 @@
       <x:c r="AA73" s="54"/>
       <x:c r="AB73" s="54"/>
       <x:c r="AC73" s="54"/>
+      <x:c r="AD73" s="81"/>
     </x:row>
     <x:row r="74" ht="28" customHeight="1">
       <x:c r="A74" s="54"/>
@@ -4236,6 +4587,7 @@
       <x:c r="AA74" s="54"/>
       <x:c r="AB74" s="54"/>
       <x:c r="AC74" s="54"/>
+      <x:c r="AD74" s="80"/>
     </x:row>
     <x:row r="75" ht="28" customHeight="1">
       <x:c r="A75" s="54"/>
@@ -4267,6 +4619,7 @@
       <x:c r="AA75" s="54"/>
       <x:c r="AB75" s="54"/>
       <x:c r="AC75" s="54"/>
+      <x:c r="AD75" s="81"/>
     </x:row>
     <x:row r="76" ht="28" customHeight="1">
       <x:c r="A76" s="54"/>
@@ -4298,6 +4651,7 @@
       <x:c r="AA76" s="54"/>
       <x:c r="AB76" s="54"/>
       <x:c r="AC76" s="54"/>
+      <x:c r="AD76" s="80"/>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
       <x:c r="A77" s="54"/>
@@ -4329,6 +4683,7 @@
       <x:c r="AA77" s="54"/>
       <x:c r="AB77" s="54"/>
       <x:c r="AC77" s="54"/>
+      <x:c r="AD77" s="81"/>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
       <x:c r="A78" s="54"/>
@@ -4360,6 +4715,7 @@
       <x:c r="AA78" s="54"/>
       <x:c r="AB78" s="54"/>
       <x:c r="AC78" s="54"/>
+      <x:c r="AD78" s="80"/>
     </x:row>
     <x:row r="79" ht="28" customHeight="1">
       <x:c r="A79" s="54"/>
@@ -4391,6 +4747,7 @@
       <x:c r="AA79" s="54"/>
       <x:c r="AB79" s="54"/>
       <x:c r="AC79" s="54"/>
+      <x:c r="AD79" s="81"/>
     </x:row>
     <x:row r="80" ht="28" customHeight="1">
       <x:c r="A80" s="54"/>
@@ -4422,6 +4779,7 @@
       <x:c r="AA80" s="54"/>
       <x:c r="AB80" s="54"/>
       <x:c r="AC80" s="54"/>
+      <x:c r="AD80" s="80"/>
     </x:row>
     <x:row r="81" ht="28" customHeight="1">
       <x:c r="A81" s="54"/>
@@ -4453,6 +4811,7 @@
       <x:c r="AA81" s="54"/>
       <x:c r="AB81" s="54"/>
       <x:c r="AC81" s="54"/>
+      <x:c r="AD81" s="81"/>
     </x:row>
     <x:row r="82" ht="28" customHeight="1">
       <x:c r="A82" s="54"/>
@@ -4484,6 +4843,7 @@
       <x:c r="AA82" s="54"/>
       <x:c r="AB82" s="54"/>
       <x:c r="AC82" s="54"/>
+      <x:c r="AD82" s="80"/>
     </x:row>
     <x:row r="83" ht="28" customHeight="1">
       <x:c r="A83" s="54"/>
@@ -4515,6 +4875,7 @@
       <x:c r="AA83" s="54"/>
       <x:c r="AB83" s="54"/>
       <x:c r="AC83" s="54"/>
+      <x:c r="AD83" s="81"/>
     </x:row>
     <x:row r="84" ht="28" customHeight="1">
       <x:c r="A84" s="54"/>
@@ -4546,6 +4907,7 @@
       <x:c r="AA84" s="54"/>
       <x:c r="AB84" s="54"/>
       <x:c r="AC84" s="54"/>
+      <x:c r="AD84" s="80"/>
     </x:row>
     <x:row r="85" ht="28" customHeight="1">
       <x:c r="A85" s="54"/>
@@ -4577,6 +4939,7 @@
       <x:c r="AA85" s="54"/>
       <x:c r="AB85" s="54"/>
       <x:c r="AC85" s="54"/>
+      <x:c r="AD85" s="81"/>
     </x:row>
     <x:row r="86" ht="28" customHeight="1">
       <x:c r="A86" s="54"/>
@@ -4608,6 +4971,7 @@
       <x:c r="AA86" s="54"/>
       <x:c r="AB86" s="54"/>
       <x:c r="AC86" s="54"/>
+      <x:c r="AD86" s="80"/>
     </x:row>
     <x:row r="87" ht="28" customHeight="1">
       <x:c r="A87" s="54"/>
@@ -4639,6 +5003,7 @@
       <x:c r="AA87" s="54"/>
       <x:c r="AB87" s="54"/>
       <x:c r="AC87" s="54"/>
+      <x:c r="AD87" s="81"/>
     </x:row>
     <x:row r="88" ht="28" customHeight="1">
       <x:c r="A88" s="54"/>
@@ -4670,6 +5035,7 @@
       <x:c r="AA88" s="54"/>
       <x:c r="AB88" s="54"/>
       <x:c r="AC88" s="54"/>
+      <x:c r="AD88" s="80"/>
     </x:row>
     <x:row r="89" ht="28" customHeight="1">
       <x:c r="A89" s="54"/>
@@ -4701,6 +5067,7 @@
       <x:c r="AA89" s="54"/>
       <x:c r="AB89" s="54"/>
       <x:c r="AC89" s="54"/>
+      <x:c r="AD89" s="81"/>
     </x:row>
     <x:row r="90" ht="28" customHeight="1">
       <x:c r="A90" s="54"/>
@@ -4732,6 +5099,7 @@
       <x:c r="AA90" s="54"/>
       <x:c r="AB90" s="54"/>
       <x:c r="AC90" s="54"/>
+      <x:c r="AD90" s="80"/>
     </x:row>
     <x:row r="91" ht="28" customHeight="1">
       <x:c r="A91" s="54"/>
@@ -4763,6 +5131,7 @@
       <x:c r="AA91" s="54"/>
       <x:c r="AB91" s="54"/>
       <x:c r="AC91" s="54"/>
+      <x:c r="AD91" s="81"/>
     </x:row>
     <x:row r="92" ht="28" customHeight="1">
       <x:c r="A92" s="54"/>
@@ -4794,6 +5163,7 @@
       <x:c r="AA92" s="54"/>
       <x:c r="AB92" s="54"/>
       <x:c r="AC92" s="54"/>
+      <x:c r="AD92" s="80"/>
     </x:row>
     <x:row r="93" ht="28" customHeight="1">
       <x:c r="A93" s="54"/>
@@ -4825,6 +5195,7 @@
       <x:c r="AA93" s="54"/>
       <x:c r="AB93" s="54"/>
       <x:c r="AC93" s="54"/>
+      <x:c r="AD93" s="81"/>
     </x:row>
     <x:row r="94" ht="28" customHeight="1">
       <x:c r="A94" s="54"/>
@@ -4856,6 +5227,7 @@
       <x:c r="AA94" s="54"/>
       <x:c r="AB94" s="54"/>
       <x:c r="AC94" s="54"/>
+      <x:c r="AD94" s="80"/>
     </x:row>
     <x:row r="95" ht="28" customHeight="1">
       <x:c r="A95" s="54"/>
@@ -4887,6 +5259,7 @@
       <x:c r="AA95" s="54"/>
       <x:c r="AB95" s="54"/>
       <x:c r="AC95" s="54"/>
+      <x:c r="AD95" s="81"/>
     </x:row>
     <x:row r="96" ht="28" customHeight="1">
       <x:c r="A96" s="54"/>
@@ -4918,6 +5291,7 @@
       <x:c r="AA96" s="54"/>
       <x:c r="AB96" s="54"/>
       <x:c r="AC96" s="54"/>
+      <x:c r="AD96" s="80"/>
     </x:row>
     <x:row r="97" ht="28" customHeight="1">
       <x:c r="A97" s="54"/>
@@ -4949,6 +5323,7 @@
       <x:c r="AA97" s="54"/>
       <x:c r="AB97" s="54"/>
       <x:c r="AC97" s="54"/>
+      <x:c r="AD97" s="81"/>
     </x:row>
     <x:row r="98" ht="28" customHeight="1">
       <x:c r="A98" s="54"/>
@@ -4980,6 +5355,7 @@
       <x:c r="AA98" s="54"/>
       <x:c r="AB98" s="54"/>
       <x:c r="AC98" s="54"/>
+      <x:c r="AD98" s="80"/>
     </x:row>
     <x:row r="99" ht="28" customHeight="1">
       <x:c r="A99" s="54"/>
@@ -5011,6 +5387,7 @@
       <x:c r="AA99" s="54"/>
       <x:c r="AB99" s="54"/>
       <x:c r="AC99" s="54"/>
+      <x:c r="AD99" s="81"/>
     </x:row>
     <x:row r="100" ht="28" customHeight="1">
       <x:c r="A100" s="54"/>
@@ -5042,6 +5419,7 @@
       <x:c r="AA100" s="54"/>
       <x:c r="AB100" s="54"/>
       <x:c r="AC100" s="54"/>
+      <x:c r="AD100" s="80"/>
     </x:row>
     <x:row r="101" ht="28" customHeight="1">
       <x:c r="A101" s="54"/>
@@ -5073,9 +5451,10 @@
       <x:c r="AA101" s="54"/>
       <x:c r="AB101" s="54"/>
       <x:c r="AC101" s="54"/>
+      <x:c r="AD101" s="81"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="3">
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="H2:H101">
       <x:formula1>"verbal,nominal"</x:formula1>
     </x:dataValidation>
@@ -5085,10 +5464,13 @@
     <x:dataValidation type="list" sqref="L2:L101">
       <x:formula1>"negated,possible,necessary,planned,future,hypothetical,conditional,questioned,reported"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="AD2:AD101">
+      <x:formula1>'Lists'!$E$2:$E$3</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf5f1202540b487a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd4ce212dad24723"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6749,7 +7131,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dddbef320cd4dca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1d125118e714e02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6762,6 +7144,7 @@
     <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -6777,6 +7160,9 @@
       <x:c r="D1" s="61" t="str">
         <x:v>rights_basis</x:v>
       </x:c>
+      <x:c r="E1" s="75" t="str">
+        <x:v>qualifier_assessed</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="62" t="str">
@@ -6791,6 +7177,9 @@
       <x:c r="D2" s="9" t="str">
         <x:v>newly_authored</x:v>
       </x:c>
+      <x:c r="E2" t="str">
+        <x:v>true</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="62" t="str">
@@ -6804,6 +7193,9 @@
       </x:c>
       <x:c r="D3" s="9" t="str">
         <x:v>public_domain</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="4">

</xml_diff>